<commit_message>
añadiendo modelos de las clases balanceadas
</commit_message>
<xml_diff>
--- a/Estimacion_error/datos_aves_marinas/2025/abril/RLOF/optimo_smape_por_clase.xlsx
+++ b/Estimacion_error/datos_aves_marinas/2025/abril/RLOF/optimo_smape_por_clase.xlsx
@@ -1,21 +1,97 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24334"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Renzo\Desktop\Data_Saiensss\Estadística\Trabajos (laborales)\BMAP\Proyectos\conteo-aves-bmap\Estimacion_error\datos_aves_marinas\2025\abril\RLOF\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93054F80-69A5-4A49-8746-0FABB215F502}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
+  <extLst>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="20">
+  <si>
+    <t>Clase</t>
+  </si>
+  <si>
+    <t>tamano_confianza</t>
+  </si>
+  <si>
+    <t>sMAPE</t>
+  </si>
+  <si>
+    <t>MAE</t>
+  </si>
+  <si>
+    <t>RMSE</t>
+  </si>
+  <si>
+    <t>n</t>
+  </si>
+  <si>
+    <t>cushuri adulto</t>
+  </si>
+  <si>
+    <t>l_0.20</t>
+  </si>
+  <si>
+    <t>pelicano adulto</t>
+  </si>
+  <si>
+    <t>m_0.20</t>
+  </si>
+  <si>
+    <t>pelicano juvenil</t>
+  </si>
+  <si>
+    <t>x_0.20</t>
+  </si>
+  <si>
+    <t>pinguino adulto</t>
+  </si>
+  <si>
+    <t>m_0.24</t>
+  </si>
+  <si>
+    <t>pinguino juvenil</t>
+  </si>
+  <si>
+    <t>l_0.34</t>
+  </si>
+  <si>
+    <t>piquero adulto</t>
+  </si>
+  <si>
+    <t>zarcillo</t>
+  </si>
+  <si>
+    <t>x_0.28</t>
+  </si>
+  <si>
+    <t>Con balanceo de clases</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -63,11 +139,68 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>161925</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>294571</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>66496</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Imagen 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2C14A66E-31DE-4BAD-B784-368EFF166B48}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="2447925"/>
+          <a:ext cx="5628571" cy="1428571"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -109,7 +242,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -141,9 +274,27 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -175,6 +326,24 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -350,52 +519,42 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F8"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:F12"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="19.140625" customWidth="1"/>
+    <col min="3" max="3" width="12.7109375" customWidth="1"/>
+    <col min="4" max="4" width="9.85546875" customWidth="1"/>
+    <col min="5" max="5" width="10.85546875" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Clase</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>tamano_confianza</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>sMAPE</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>MAE</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>RMSE</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>n</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>cushuri adulto</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>l_0.20</t>
-        </is>
+    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" t="s">
+        <v>7</v>
       </c>
       <c r="C2">
         <v>200</v>
@@ -410,16 +569,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>pelicano adulto</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>m_0.20</t>
-        </is>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" t="s">
+        <v>9</v>
       </c>
       <c r="C3">
         <v>66.67</v>
@@ -434,40 +589,32 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>pelicano juvenil</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>x_0.20</t>
-        </is>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" t="s">
+        <v>11</v>
       </c>
       <c r="C4">
-        <v>81.90000000000001</v>
+        <v>81.900000000000006</v>
       </c>
       <c r="D4">
         <v>1.6</v>
       </c>
       <c r="E4">
-        <v>2.449</v>
+        <v>2.4489999999999998</v>
       </c>
       <c r="F4">
         <v>5</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>pinguino adulto</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>m_0.24</t>
-        </is>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" t="s">
+        <v>13</v>
       </c>
       <c r="C5">
         <v>57.4</v>
@@ -476,28 +623,24 @@
         <v>1.333</v>
       </c>
       <c r="E5">
-        <v>1.826</v>
+        <v>1.8260000000000001</v>
       </c>
       <c r="F5">
         <v>15</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>pinguino juvenil</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>l_0.34</t>
-        </is>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" t="s">
+        <v>15</v>
       </c>
       <c r="C6">
         <v>124.03</v>
       </c>
       <c r="D6">
-        <v>3.333</v>
+        <v>3.3330000000000002</v>
       </c>
       <c r="E6">
         <v>5.077</v>
@@ -506,16 +649,12 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>piquero adulto</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>l_0.20</t>
-        </is>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" t="s">
+        <v>7</v>
       </c>
       <c r="C7">
         <v>200</v>
@@ -530,16 +669,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>zarcillo</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>x_0.28</t>
-        </is>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" t="s">
+        <v>18</v>
       </c>
       <c r="C8">
         <v>13.36</v>
@@ -548,13 +683,19 @@
         <v>2.609</v>
       </c>
       <c r="E8">
-        <v>3.414</v>
+        <v>3.4140000000000001</v>
       </c>
       <c r="F8">
         <v>23</v>
       </c>
     </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>19</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>